<commit_message>
semi working scraping with data extraction table
</commit_message>
<xml_diff>
--- a/BOOKING_RESULT_Brasov_05-15-2026_000000_07-20-2026_000000_3_guests.xlsx
+++ b/BOOKING_RESULT_Brasov_05-15-2026_000000_07-20-2026_000000_3_guests.xlsx
@@ -19,241 +19,295 @@
     <x:t>HotelName</x:t>
   </x:si>
   <x:si>
-    <x:t>Url</x:t>
+    <x:t>HotelUrl</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Rating</x:t>
   </x:si>
   <x:si>
     <x:t>Price</x:t>
   </x:si>
   <x:si>
-    <x:t>Rating</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Central houses budget friendly</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/central-houses-budget-friendly.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuALrrKDKBsACAdICJDNkMWFmYTZkLWJhN2UtNDE5MS04NmIwLTAxNjk5OTM2NmQzMNgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-01-07&amp;checkout=2026-01-10&amp;dest_id=-1153951&amp;dest_type=city&amp;group_adults=2&amp;req_adults=2&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=1&amp;hapos=1&amp;sr_order=popularity&amp;srpvid=304c7af7f14d7d22b74caeec5251d628&amp;srepoch=1766488749&amp;all_sr_blocks=1407467402_412519025_0_0_0&amp;highlighted_blocks=1407467402_412519025_0_0_0&amp;matching_block_id=1407467402_412519025_0_0_0&amp;sr_pri_blocks=1407467402_412519025_0_0_0__70206&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>702 lei</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8.0</x:t>
-  </x:si>
-  <x:si>
-    <x:t>YamaLuxe Luxury Apartments - București</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/yamaluxe-apartments-bucuresti.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuALrrKDKBsACAdICJDNkMWFmYTZkLWJhN2UtNDE5MS04NmIwLTAxNjk5OTM2NmQzMNgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-01-07&amp;checkout=2026-01-10&amp;dest_id=-1153951&amp;dest_type=city&amp;group_adults=2&amp;req_adults=2&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=2&amp;hapos=2&amp;sr_order=popularity&amp;srpvid=304c7af7f14d7d22b74caeec5251d628&amp;srepoch=1766488749&amp;all_sr_blocks=1171951105_389727277_2_2_0&amp;highlighted_blocks=1171951105_389727277_2_2_0&amp;matching_block_id=1171951105_389727277_2_2_0&amp;sr_pri_blocks=1171951105_389727277_2_2_0__61435&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t/>
+    <x:t>https://www.booking.com/hotel/ro/white-residence-brasov.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuAK0qKrKBsACAdICJDA3Yjg3ODMzLWFlNmYtNDVmMi04NDkwLWQyOWNlZDU1NTgyYtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=1&amp;hapos=1&amp;sr_order=popularity&amp;srpvid=f0df5c6391330050&amp;srepoch=1766495350&amp;all_sr_blocks=559451708_209413944_0_0_0&amp;highlighted_blocks=559451708_209413944_0_0_0&amp;matching_block_id=559451708_209413944_0_0_0&amp;sr_pri_blocks=559451708_209413944_0_0_0__1537547&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MGI studio CORESI &amp; parking</x:t>
+  </x:si>
+  <x:si>
+    <x:t>15,375 lei</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11,193 lei</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9.3</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Bark Inn - Bed and Breakfast</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/bark-inn-bed-and-breakfast.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuAK0qKrKBsACAdICJDA3Yjg3ODMzLWFlNmYtNDVmMi04NDkwLWQyOWNlZDU1NTgyYtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=3&amp;hapos=3&amp;sr_order=popularity&amp;srpvid=f0df5c6391330050&amp;srepoch=1766495350&amp;all_sr_blocks=1320902003_404782112_0_1_0&amp;highlighted_blocks=1320902003_404782112_0_1_0&amp;matching_block_id=1320902003_404782112_0_1_0&amp;sr_pri_blocks=1320902003_404782112_0_1_0__3046050&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9.2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>51,879 lei</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Apartament Racadau</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/apartament-racadau-brasov.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuAK0qKrKBsACAdICJDA3Yjg3ODMzLWFlNmYtNDVmMi04NDkwLWQyOWNlZDU1NTgyYtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=4&amp;hapos=4&amp;sr_order=popularity&amp;srpvid=f0df5c6391330050&amp;srepoch=1766495350&amp;all_sr_blocks=749019701_331158284_3_0_0&amp;highlighted_blocks=749019701_331158284_3_0_0&amp;matching_block_id=749019701_331158284_3_0_0&amp;sr_pri_blocks=749019701_331158284_3_0_0__1488816&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9.8</x:t>
+  </x:si>
+  <x:si>
+    <x:t>19,279 lei</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KOA - Aparthotel</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/koa-aparthotel-1.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuAK0qKrKBsACAdICJDA3Yjg3ODMzLWFlNmYtNDVmMi04NDkwLWQyOWNlZDU1NTgyYtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=5&amp;hapos=5&amp;sr_order=popularity&amp;srpvid=f0df5c6391330050&amp;srepoch=1766495350&amp;all_sr_blocks=995130006_405288024_4_0_0&amp;highlighted_blocks=995130006_405288024_4_0_0&amp;matching_block_id=995130006_405288024_4_0_0&amp;sr_pri_blocks=995130006_405288024_4_0_0__3084939&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9.6</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Select City Center Apartments</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/historical-center-apartment.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuAK0qKrKBsACAdICJDA3Yjg3ODMzLWFlNmYtNDVmMi04NDkwLWQyOWNlZDU1NTgyYtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=6&amp;hapos=6&amp;sr_order=popularity&amp;srpvid=f0df5c6391330050&amp;srepoch=1766495350&amp;all_sr_blocks=31850708_421755992_3_0_0&amp;highlighted_blocks=31850708_421755992_3_0_0&amp;matching_block_id=31850708_421755992_3_0_0&amp;sr_pri_blocks=31850708_421755992_3_0_0__2585682&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>25,857 lei</x:t>
+  </x:si>
+  <x:si>
+    <x:t>36,050 lei</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Pension Bavaria</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/pension-bavaria.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuAK0qKrKBsACAdICJDA3Yjg3ODMzLWFlNmYtNDVmMi04NDkwLWQyOWNlZDU1NTgyYtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=7&amp;hapos=7&amp;sr_order=popularity&amp;srpvid=f0df5c6391330050&amp;srepoch=1766495350&amp;all_sr_blocks=31458704_246256401_3_0_0&amp;highlighted_blocks=31458704_246256401_3_0_0&amp;matching_block_id=31458704_246256401_3_0_0&amp;sr_pri_blocks=31458704_246256401_3_0_0__1971000&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>19,710 lei</x:t>
+  </x:si>
+  <x:si>
+    <x:t>73,128 lei</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TampaView ApartHotel</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/tampaview-aparthotel.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuAK0qKrKBsACAdICJDA3Yjg3ODMzLWFlNmYtNDVmMi04NDkwLWQyOWNlZDU1NTgyYtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=8&amp;hapos=8&amp;sr_order=popularity&amp;srpvid=f0df5c6391330050&amp;srepoch=1766495350&amp;all_sr_blocks=1422457001_423999646_0_0_0&amp;highlighted_blocks=1422457001_423999646_0_0_0&amp;matching_block_id=1422457001_423999646_0_0_0&amp;sr_pri_blocks=1422457001_423999646_0_0_0__3605000&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9.9</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Luca</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/luca-brasov2.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuAK0qKrKBsACAdICJDA3Yjg3ODMzLWFlNmYtNDVmMi04NDkwLWQyOWNlZDU1NTgyYtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=9&amp;hapos=9&amp;sr_order=popularity&amp;srpvid=f0df5c6391330050&amp;srepoch=1766495350&amp;all_sr_blocks=1348675301_408707859_0_0_0&amp;highlighted_blocks=1348675301_408707859_0_0_0&amp;matching_block_id=1348675301_408707859_0_0_0&amp;sr_pri_blocks=1348675301_408707859_0_0_0__1287000&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>12,870 lei</x:t>
+  </x:si>
+  <x:si>
+    <x:t>21,853 lei</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KOA - Davino Aparthotel</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/koa-davino-aparthotel.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuAK0qKrKBsACAdICJDA3Yjg3ODMzLWFlNmYtNDVmMi04NDkwLWQyOWNlZDU1NTgyYtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=10&amp;hapos=10&amp;sr_order=popularity&amp;srpvid=f0df5c6391330050&amp;srepoch=1766495350&amp;all_sr_blocks=1094405206_382349208_4_0_0_877326&amp;highlighted_blocks=1094405206_382349208_4_0_0_877326&amp;matching_block_id=1094405206_382349208_4_0_0_877326&amp;sr_pri_blocks=1094405206_382349208_4_0_0_877326_2571956&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>25,720 lei</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KOA - Nest</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/koa-nest-brasov20.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuAK0qKrKBsACAdICJDA3Yjg3ODMzLWFlNmYtNDVmMi04NDkwLWQyOWNlZDU1NTgyYtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=11&amp;hapos=11&amp;sr_order=popularity&amp;srpvid=f0df5c6391330050&amp;srepoch=1766495350&amp;all_sr_blocks=1324188501_425784292_4_0_0&amp;highlighted_blocks=1324188501_425784292_4_0_0&amp;matching_block_id=1324188501_425784292_4_0_0&amp;sr_pri_blocks=1324188501_425784292_4_0_0__4051944&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9.7</x:t>
+  </x:si>
+  <x:si>
+    <x:t>JAD Luxury Apartments Kasper</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/jad-confortable-promenada-coresi.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuAK0qKrKBsACAdICJDA3Yjg3ODMzLWFlNmYtNDVmMi04NDkwLWQyOWNlZDU1NTgyYtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=12&amp;hapos=12&amp;sr_order=popularity&amp;srpvid=f0df5c6391330050&amp;srepoch=1766495350&amp;all_sr_blocks=1109165407_383666009_3_0_0_337045&amp;highlighted_blocks=1109165407_383666009_3_0_0_337045&amp;matching_block_id=1109165407_383666009_3_0_0_337045&amp;sr_pri_blocks=1109165407_383666009_3_0_0_337045_2323200&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9.5</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9.1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KOA - Memo Haus</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/koa-memo-haus.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuAK0qKrKBsACAdICJDA3Yjg3ODMzLWFlNmYtNDVmMi04NDkwLWQyOWNlZDU1NTgyYtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=13&amp;hapos=13&amp;sr_order=popularity&amp;srpvid=f0df5c6391330050&amp;srepoch=1766495350&amp;all_sr_blocks=1395631202_411470735_4_0_0&amp;highlighted_blocks=1395631202_411470735_4_0_0&amp;matching_block_id=1395631202_411470735_4_0_0&amp;sr_pri_blocks=1395631202_411470735_4_0_0__3344279&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8.8</x:t>
+  </x:si>
+  <x:si>
+    <x:t>31,321 lei</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Skylark Central Aparthotel</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/skylark-geneva-suite-with-fireplace-amp-view.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuAK0qKrKBsACAdICJDA3Yjg3ODMzLWFlNmYtNDVmMi04NDkwLWQyOWNlZDU1NTgyYtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=14&amp;hapos=14&amp;sr_order=popularity&amp;srpvid=f0df5c6391330050&amp;srepoch=1766495350&amp;all_sr_blocks=1117857507_384637893_3_0_0&amp;highlighted_blocks=1117857507_384637893_3_0_0&amp;matching_block_id=1117857507_384637893_3_0_0&amp;sr_pri_blocks=1117857507_384637893_3_0_0__3465000&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>34,650 lei</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PEAK Aparthotel - Old Town - by CityHost</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/peak-aparthotel-by-cityhost.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuAK0qKrKBsACAdICJDA3Yjg3ODMzLWFlNmYtNDVmMi04NDkwLWQyOWNlZDU1NTgyYtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=15&amp;hapos=15&amp;sr_order=popularity&amp;srpvid=f0df5c6391330050&amp;srepoch=1766495350&amp;all_sr_blocks=1166912003_389307937_3_0_0&amp;highlighted_blocks=1166912003_389307937_3_0_0&amp;matching_block_id=1166912003_389307937_3_0_0&amp;sr_pri_blocks=1166912003_389307937_3_0_0__2975419&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>33,044 lei29,754 lei</x:t>
+  </x:si>
+  <x:si>
+    <x:t>JAD Comfortable Apartments</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/jad-isaran.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuAK0qKrKBsACAdICJDA3Yjg3ODMzLWFlNmYtNDVmMi04NDkwLWQyOWNlZDU1NTgyYtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=16&amp;hapos=16&amp;sr_order=popularity&amp;srpvid=f0df5c6391330050&amp;srepoch=1766495350&amp;all_sr_blocks=969942706_369395472_3_0_0_337069&amp;highlighted_blocks=969942706_369395472_3_0_0_337069&amp;matching_block_id=969942706_369395472_3_0_0_337069&amp;sr_pri_blocks=969942706_369395472_3_0_0_337069_2185260&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9.4</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Casa Roth</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/casa-roth-apartments.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuAK0qKrKBsACAdICJDA3Yjg3ODMzLWFlNmYtNDVmMi04NDkwLWQyOWNlZDU1NTgyYtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=17&amp;hapos=17&amp;sr_order=popularity&amp;srpvid=f0df5c6391330050&amp;srepoch=1766495350&amp;all_sr_blocks=251825904_222711381_3_0_0&amp;highlighted_blocks=251825904_222711381_3_0_0&amp;matching_block_id=251825904_222711381_3_0_0&amp;sr_pri_blocks=251825904_222711381_3_0_0__1927930&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8.1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Pensiunea Leo</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/pensiunea-leo.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuAK0qKrKBsACAdICJDA3Yjg3ODMzLWFlNmYtNDVmMi04NDkwLWQyOWNlZDU1NTgyYtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=18&amp;hapos=18&amp;sr_order=popularity&amp;srpvid=f0df5c6391330050&amp;srepoch=1766495350&amp;all_sr_blocks=34116103_264837064_3_0_0&amp;highlighted_blocks=34116103_264837064_3_0_0&amp;matching_block_id=34116103_264837064_3_0_0&amp;sr_pri_blocks=34116103_264837064_3_0_0__2178000&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>21,780 lei</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Mandala Designer Apartments with Free Private Parking, near Mall Coresi</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/mandala-a-designer-penthouse-with-free-private-parking-near-mall-coresi.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuAK0qKrKBsACAdICJDA3Yjg3ODMzLWFlNmYtNDVmMi04NDkwLWQyOWNlZDU1NTgyYtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=19&amp;hapos=19&amp;sr_order=popularity&amp;srpvid=f0df5c6391330050&amp;srepoch=1766495350&amp;all_sr_blocks=929406402_364926508_5_0_0&amp;highlighted_blocks=929406402_364926508_5_0_0&amp;matching_block_id=929406402_364926508_5_0_0&amp;sr_pri_blocks=929406402_364926508_5_0_0__7312800&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KOA - Sunlight Apartment</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/sunlight-apartment-by-taboo.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuAK0qKrKBsACAdICJDA3Yjg3ODMzLWFlNmYtNDVmMi04NDkwLWQyOWNlZDU1NTgyYtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=20&amp;hapos=20&amp;sr_order=popularity&amp;srpvid=f0df5c6391330050&amp;srepoch=1766495350&amp;all_sr_blocks=806763501_360416925_4_0_0&amp;highlighted_blocks=806763501_360416925_4_0_0&amp;matching_block_id=806763501_360416925_4_0_0&amp;sr_pri_blocks=806763501_360416925_4_0_0__2564430&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>25,644 lei</x:t>
   </x:si>
   <x:si>
     <x:t>9.0</x:t>
   </x:si>
   <x:si>
-    <x:t>Bucharest Central C Apartment</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/old-town-bohemian-attic.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuALrrKDKBsACAdICJDNkMWFmYTZkLWJhN2UtNDE5MS04NmIwLTAxNjk5OTM2NmQzMNgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-01-07&amp;checkout=2026-01-10&amp;dest_id=-1153951&amp;dest_type=city&amp;group_adults=2&amp;req_adults=2&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=3&amp;hapos=3&amp;sr_order=popularity&amp;srpvid=304c7af7f14d7d22b74caeec5251d628&amp;srepoch=1766488749&amp;all_sr_blocks=1052035601_399555355_2_0_0&amp;highlighted_blocks=1052035601_399555355_2_0_0&amp;matching_block_id=1052035601_399555355_2_0_0&amp;sr_pri_blocks=1052035601_399555355_2_0_0__62428&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>624 lei</x:t>
+    <x:t>Bb's Cosy Apartments</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/bb-39-s-cosy-apartments-brasov.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuAK0qKrKBsACAdICJDA3Yjg3ODMzLWFlNmYtNDVmMi04NDkwLWQyOWNlZDU1NTgyYtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=21&amp;hapos=21&amp;sr_order=popularity&amp;srpvid=f0df5c6391330050&amp;srepoch=1766495350&amp;all_sr_blocks=295908503_329654120_0_0_0&amp;highlighted_blocks=295908503_329654120_0_0_0&amp;matching_block_id=295908503_329654120_0_0_0&amp;sr_pri_blocks=295908503_329654120_0_0_0__2194500&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>25,080 lei21,945 lei</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8.3</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Warm Amber Suites Brașov</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/cosmopolit-lifestyle.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuAK0qKrKBsACAdICJDA3Yjg3ODMzLWFlNmYtNDVmMi04NDkwLWQyOWNlZDU1NTgyYtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=22&amp;hapos=22&amp;sr_order=popularity&amp;srpvid=f0df5c6391330050&amp;srepoch=1766495350&amp;all_sr_blocks=282931413_126032420_3_0_0_677855&amp;highlighted_blocks=282931413_126032420_3_0_0_677855&amp;matching_block_id=282931413_126032420_3_0_0_677855&amp;sr_pri_blocks=282931413_126032420_3_0_0_677855_3132080&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Coresi Mall Area Studios &amp; Apartments by GLAM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/coresi-mall-area-studios-amp-apartments-by-glam.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuAK0qKrKBsACAdICJDA3Yjg3ODMzLWFlNmYtNDVmMi04NDkwLWQyOWNlZDU1NTgyYtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=23&amp;hapos=23&amp;sr_order=popularity&amp;srpvid=f0df5c6391330050&amp;srepoch=1766495350&amp;all_sr_blocks=1118248102_412223809_3_0_0&amp;highlighted_blocks=1118248102_412223809_3_0_0&amp;matching_block_id=1118248102_412223809_3_0_0&amp;sr_pri_blocks=1118248102_412223809_3_0_0__2877300&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>28,773 lei</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8.6</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Old Town View &amp; Balcony Apartments MM Host</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/brasov-old-town-with-mountain-view.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuAK0qKrKBsACAdICJDA3Yjg3ODMzLWFlNmYtNDVmMi04NDkwLWQyOWNlZDU1NTgyYtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=24&amp;hapos=24&amp;sr_order=popularity&amp;srpvid=f0df5c6391330050&amp;srepoch=1766495350&amp;all_sr_blocks=1428222201_417107964_3_0_0&amp;highlighted_blocks=1428222201_417107964_3_0_0&amp;matching_block_id=1428222201_417107964_3_0_0&amp;sr_pri_blocks=1428222201_417107964_3_0_0__5187930&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>18,993 lei16,263 lei</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Main Square Apartments &amp; More</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/main-square-apartments-amp-more.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuAK0qKrKBsACAdICJDA3Yjg3ODMzLWFlNmYtNDVmMi04NDkwLWQyOWNlZDU1NTgyYtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=25&amp;hapos=25&amp;sr_order=popularity&amp;srpvid=f0df5c6391330050&amp;srepoch=1766495350&amp;all_sr_blocks=116190210_208743329_0_0_0&amp;highlighted_blocks=116190210_208743329_0_0_0&amp;matching_block_id=116190210_208743329_0_0_0&amp;sr_pri_blocks=116190210_208743329_0_0_0__1626341&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>7.5</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Città Studi Suites - Top Collection</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/it/bb-too-cute-2b-str8.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuAKRoarKBsACAdICJDZmMGU5Mzc2LTJjYjgtNGRiMy05NWI0LWRhYmUwZjRkYzUzYtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-08-10&amp;checkout=2026-08-15&amp;dest_id=-121726&amp;dest_type=city&amp;group_adults=1&amp;req_adults=1&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=26&amp;hapos=26&amp;sr_order=popularity&amp;srpvid=d0bf5a9436ca15d7&amp;srepoch=1766494379&amp;all_sr_blocks=120214214_373646928_1_0_0&amp;highlighted_blocks=120214214_373646928_1_0_0&amp;matching_block_id=120214214_373646928_1_0_0&amp;sr_pri_blocks=120214214_373646928_1_0_0__43850&amp;from=searchresults</x:t>
   </x:si>
   <x:si>
     <x:t>8.9</x:t>
   </x:si>
   <x:si>
-    <x:t>Piața Romană Zone Apartament</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/piata-romana-zone-apartament.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuALrrKDKBsACAdICJDNkMWFmYTZkLWJhN2UtNDE5MS04NmIwLTAxNjk5OTM2NmQzMNgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-01-07&amp;checkout=2026-01-10&amp;dest_id=-1153951&amp;dest_type=city&amp;group_adults=2&amp;req_adults=2&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=4&amp;hapos=4&amp;sr_order=popularity&amp;srpvid=304c7af7f14d7d22b74caeec5251d628&amp;srepoch=1766488749&amp;all_sr_blocks=1517819701_423491097_2_0_0&amp;highlighted_blocks=1517819701_423491097_2_0_0&amp;matching_block_id=1517819701_423491097_2_0_0&amp;sr_pri_blocks=1517819701_423491097_2_0_0__59700&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9.5</x:t>
-  </x:si>
-  <x:si>
-    <x:t>The City Retreat Apart-Hotel</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/the-city-retreat-apart.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuALrrKDKBsACAdICJDNkMWFmYTZkLWJhN2UtNDE5MS04NmIwLTAxNjk5OTM2NmQzMNgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-01-07&amp;checkout=2026-01-10&amp;dest_id=-1153951&amp;dest_type=city&amp;group_adults=2&amp;req_adults=2&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=5&amp;hapos=5&amp;sr_order=popularity&amp;srpvid=304c7af7f14d7d22b74caeec5251d628&amp;srepoch=1766488749&amp;all_sr_blocks=1332711703_405777882_2_0_0_913798&amp;highlighted_blocks=1332711703_405777882_2_0_0_913798&amp;matching_block_id=1332711703_405777882_2_0_0_913798&amp;sr_pri_blocks=1332711703_405777882_2_0_0_913798_76837&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>768 lei</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8.6</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Old City Calea Victoriei Deluxe</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/old-city-calea-victoriei-deluxe.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuALrrKDKBsACAdICJDNkMWFmYTZkLWJhN2UtNDE5MS04NmIwLTAxNjk5OTM2NmQzMNgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-01-07&amp;checkout=2026-01-10&amp;dest_id=-1153951&amp;dest_type=city&amp;group_adults=2&amp;req_adults=2&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=6&amp;hapos=6&amp;sr_order=popularity&amp;srpvid=304c7af7f14d7d22b74caeec5251d628&amp;srepoch=1766488749&amp;all_sr_blocks=1504909701_422237916_2_0_0&amp;highlighted_blocks=1504909701_422237916_2_0_0&amp;matching_block_id=1504909701_422237916_2_0_0&amp;sr_pri_blocks=1504909701_422237916_2_0_0__76150&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9.6</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Home Guest - Apartment 3</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/home-guest-apartments-bucuresti1.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuALrrKDKBsACAdICJDNkMWFmYTZkLWJhN2UtNDE5MS04NmIwLTAxNjk5OTM2NmQzMNgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-01-07&amp;checkout=2026-01-10&amp;dest_id=-1153951&amp;dest_type=city&amp;group_adults=2&amp;req_adults=2&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=7&amp;hapos=7&amp;sr_order=popularity&amp;srpvid=304c7af7f14d7d22b74caeec5251d628&amp;srepoch=1766488749&amp;all_sr_blocks=1385508701_414901259_2_0_0&amp;highlighted_blocks=1385508701_414901259_2_0_0&amp;matching_block_id=1385508701_414901259_2_0_0&amp;sr_pri_blocks=1385508701_414901259_2_0_0__45900&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>7.5</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Central Residence Apartment 812 B3</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/central-residence-apartment-812.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuALrrKDKBsACAdICJDNkMWFmYTZkLWJhN2UtNDE5MS04NmIwLTAxNjk5OTM2NmQzMNgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-01-07&amp;checkout=2026-01-10&amp;dest_id=-1153951&amp;dest_type=city&amp;group_adults=2&amp;req_adults=2&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=8&amp;hapos=8&amp;sr_order=popularity&amp;srpvid=304c7af7f14d7d22b74caeec5251d628&amp;srepoch=1766488749&amp;all_sr_blocks=1144452501_387298811_2_0_0_561427&amp;highlighted_blocks=1144452501_387298811_2_0_0_561427&amp;matching_block_id=1144452501_387298811_2_0_0_561427&amp;sr_pri_blocks=1144452501_387298811_2_0_0_561427_62000&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>620 lei</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9.3</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Arena Park</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/arena-park.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuALrrKDKBsACAdICJDNkMWFmYTZkLWJhN2UtNDE5MS04NmIwLTAxNjk5OTM2NmQzMNgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-01-07&amp;checkout=2026-01-10&amp;dest_id=-1153951&amp;dest_type=city&amp;group_adults=2&amp;req_adults=2&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=9&amp;hapos=9&amp;sr_order=popularity&amp;srpvid=304c7af7f14d7d22b74caeec5251d628&amp;srepoch=1766488749&amp;all_sr_blocks=1392496305_411201441_2_0_0_1164546&amp;highlighted_blocks=1392496305_411201441_2_0_0_1164546&amp;matching_block_id=1392496305_411201441_2_0_0_1164546&amp;sr_pri_blocks=1392496305_411201441_2_0_0_1164546_67500&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Central Residence Studio P25</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/central-residence-studio-p25.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuALrrKDKBsACAdICJDNkMWFmYTZkLWJhN2UtNDE5MS04NmIwLTAxNjk5OTM2NmQzMNgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-01-07&amp;checkout=2026-01-10&amp;dest_id=-1153951&amp;dest_type=city&amp;group_adults=2&amp;req_adults=2&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=10&amp;hapos=10&amp;sr_order=popularity&amp;srpvid=304c7af7f14d7d22b74caeec5251d628&amp;srepoch=1766488749&amp;all_sr_blocks=1268463001_399568933_2_0_0_603269&amp;highlighted_blocks=1268463001_399568933_2_0_0_603269&amp;matching_block_id=1268463001_399568933_2_0_0_603269&amp;sr_pri_blocks=1268463001_399568933_2_0_0_603269_62000&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AT Central Apartments</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/at-central-apartments.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuALrrKDKBsACAdICJDNkMWFmYTZkLWJhN2UtNDE5MS04NmIwLTAxNjk5OTM2NmQzMNgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-01-07&amp;checkout=2026-01-10&amp;dest_id=-1153951&amp;dest_type=city&amp;group_adults=2&amp;req_adults=2&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=11&amp;hapos=11&amp;sr_order=popularity&amp;srpvid=304c7af7f14d7d22b74caeec5251d628&amp;srepoch=1766488749&amp;all_sr_blocks=503858904_408972632_2_0_0_521942&amp;highlighted_blocks=503858904_408972632_2_0_0_521942&amp;matching_block_id=503858904_408972632_2_0_0_521942&amp;sr_pri_blocks=503858904_408972632_2_0_0_521942_96000&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>960 lei</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9.2</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Pura Vida Downtown Tiny houses</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/downtown-tiny-houses-near-cismigiu-gardens.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuALrrKDKBsACAdICJDNkMWFmYTZkLWJhN2UtNDE5MS04NmIwLTAxNjk5OTM2NmQzMNgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-01-07&amp;checkout=2026-01-10&amp;dest_id=-1153951&amp;dest_type=city&amp;group_adults=2&amp;req_adults=2&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=12&amp;hapos=12&amp;sr_order=popularity&amp;srpvid=304c7af7f14d7d22b74caeec5251d628&amp;srepoch=1766488749&amp;all_sr_blocks=1289267905_401875389_2_0_0_750797&amp;highlighted_blocks=1289267905_401875389_2_0_0_750797&amp;matching_block_id=1289267905_401875389_2_0_0_750797&amp;sr_pri_blocks=1289267905_401875389_2_0_0_750797_57335&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>573 lei</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8.4</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Upground Residence Apartments</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/upground-residence-apartments.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuALrrKDKBsACAdICJDNkMWFmYTZkLWJhN2UtNDE5MS04NmIwLTAxNjk5OTM2NmQzMNgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-01-07&amp;checkout=2026-01-10&amp;dest_id=-1153951&amp;dest_type=city&amp;group_adults=2&amp;req_adults=2&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=13&amp;hapos=13&amp;sr_order=popularity&amp;srpvid=304c7af7f14d7d22b74caeec5251d628&amp;srepoch=1766488749&amp;all_sr_blocks=460874901_0_2_0_0&amp;highlighted_blocks=460874901_0_2_0_0&amp;matching_block_id=460874901_0_2_0_0&amp;sr_pri_blocks=460874901_0_2_0_0__84302&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>365 Apartments in Bucharest</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/365-apartments-in-bucharest.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuALrrKDKBsACAdICJDNkMWFmYTZkLWJhN2UtNDE5MS04NmIwLTAxNjk5OTM2NmQzMNgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-01-07&amp;checkout=2026-01-10&amp;dest_id=-1153951&amp;dest_type=city&amp;group_adults=2&amp;req_adults=2&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=14&amp;hapos=14&amp;sr_order=popularity&amp;srpvid=304c7af7f14d7d22b74caeec5251d628&amp;srepoch=1766488749&amp;all_sr_blocks=1089796301_381884070_2_0_0&amp;highlighted_blocks=1089796301_381884070_2_0_0&amp;matching_block_id=1089796301_381884070_2_0_0&amp;sr_pri_blocks=1089796301_381884070_2_0_0__121784&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8.8</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Riviera Unirii Residence</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/riviera-unirii-residence.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuALrrKDKBsACAdICJDNkMWFmYTZkLWJhN2UtNDE5MS04NmIwLTAxNjk5OTM2NmQzMNgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-01-07&amp;checkout=2026-01-10&amp;dest_id=-1153951&amp;dest_type=city&amp;group_adults=2&amp;req_adults=2&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=15&amp;hapos=15&amp;sr_order=popularity&amp;srpvid=304c7af7f14d7d22b74caeec5251d628&amp;srepoch=1766488749&amp;all_sr_blocks=927007703_383045109_0_2_0&amp;highlighted_blocks=927007703_383045109_0_2_0&amp;matching_block_id=927007703_383045109_0_2_0&amp;sr_pri_blocks=927007703_383045109_0_2_0__57000&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8.1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Crystal Palace Hotel</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/crystal-palace.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuALrrKDKBsACAdICJDNkMWFmYTZkLWJhN2UtNDE5MS04NmIwLTAxNjk5OTM2NmQzMNgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-01-07&amp;checkout=2026-01-10&amp;dest_id=-1153951&amp;dest_type=city&amp;group_adults=2&amp;req_adults=2&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=16&amp;hapos=16&amp;sr_order=popularity&amp;srpvid=304c7af7f14d7d22b74caeec5251d628&amp;srepoch=1766488749&amp;all_sr_blocks=4116105_141318468_2_2_0_590627&amp;highlighted_blocks=4116105_141318468_2_2_0_590627&amp;matching_block_id=4116105_141318468_2_2_0_590627&amp;sr_pri_blocks=4116105_141318468_2_2_0_590627_167642&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9.1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Ultimate Living Experience - Modern Accommodation &amp; Free Parking near Romexpo</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/two-bedroom-apartment-with-free-parking.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuALrrKDKBsACAdICJDNkMWFmYTZkLWJhN2UtNDE5MS04NmIwLTAxNjk5OTM2NmQzMNgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-01-07&amp;checkout=2026-01-10&amp;dest_id=-1153951&amp;dest_type=city&amp;group_adults=2&amp;req_adults=2&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=17&amp;hapos=17&amp;sr_order=popularity&amp;srpvid=304c7af7f14d7d22b74caeec5251d628&amp;srepoch=1766488749&amp;all_sr_blocks=769352802_334675763_2_0_0&amp;highlighted_blocks=769352802_334675763_2_0_0&amp;matching_block_id=769352802_334675763_2_0_0&amp;sr_pri_blocks=769352802_334675763_2_0_0__93670&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>937 lei</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HIGHLINE DOWNTOWN ApartHotel OLDTOWN UNIRII SQUARE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/highline-downtown.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuALrrKDKBsACAdICJDNkMWFmYTZkLWJhN2UtNDE5MS04NmIwLTAxNjk5OTM2NmQzMNgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-01-07&amp;checkout=2026-01-10&amp;dest_id=-1153951&amp;dest_type=city&amp;group_adults=2&amp;req_adults=2&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=18&amp;hapos=18&amp;sr_order=popularity&amp;srpvid=304c7af7f14d7d22b74caeec5251d628&amp;srepoch=1766488749&amp;all_sr_blocks=550833714_200909667_2_0_0&amp;highlighted_blocks=550833714_200909667_2_0_0&amp;matching_block_id=550833714_200909667_2_0_0&amp;sr_pri_blocks=550833714_200909667_2_0_0__104438&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1,044 lei</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8.7</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Downtown Terrace Nest Victoriei Gara de Nord</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/downtown-terrace-nest-victory-gara-de-nord.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuALrrKDKBsACAdICJDNkMWFmYTZkLWJhN2UtNDE5MS04NmIwLTAxNjk5OTM2NmQzMNgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-01-07&amp;checkout=2026-01-10&amp;dest_id=-1153951&amp;dest_type=city&amp;group_adults=2&amp;req_adults=2&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=19&amp;hapos=19&amp;sr_order=popularity&amp;srpvid=304c7af7f14d7d22b74caeec5251d628&amp;srepoch=1766488749&amp;all_sr_blocks=1470621701_418410430_2_0_0&amp;highlighted_blocks=1470621701_418410430_2_0_0&amp;matching_block_id=1470621701_418410430_2_0_0&amp;sr_pri_blocks=1470621701_418410430_2_0_0__173400&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>One by One - by Grand Accommodation</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/bucharest-check-in.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuALrrKDKBsACAdICJDNkMWFmYTZkLWJhN2UtNDE5MS04NmIwLTAxNjk5OTM2NmQzMNgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-01-07&amp;checkout=2026-01-10&amp;dest_id=-1153951&amp;dest_type=city&amp;group_adults=2&amp;req_adults=2&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=20&amp;hapos=20&amp;sr_order=popularity&amp;srpvid=304c7af7f14d7d22b74caeec5251d628&amp;srepoch=1766488749&amp;all_sr_blocks=224642942_413845015_2_0_0&amp;highlighted_blocks=224642942_413845015_2_0_0&amp;matching_block_id=224642942_413845015_2_0_0&amp;sr_pri_blocks=224642942_413845015_2_0_0__108000&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Wonderful Apartments in Prime North Location - Heaven for Extended Stays</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/wonderful-1br-amp-balcony-heaven-for-extended-stays.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuALrrKDKBsACAdICJDNkMWFmYTZkLWJhN2UtNDE5MS04NmIwLTAxNjk5OTM2NmQzMNgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-01-07&amp;checkout=2026-01-10&amp;dest_id=-1153951&amp;dest_type=city&amp;group_adults=2&amp;req_adults=2&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=21&amp;hapos=21&amp;sr_order=popularity&amp;srpvid=304c7af7f14d7d22b74caeec5251d628&amp;srepoch=1766488749&amp;all_sr_blocks=1061440001_378456007_2_0_0&amp;highlighted_blocks=1061440001_378456007_2_0_0&amp;matching_block_id=1061440001_378456007_2_0_0&amp;sr_pri_blocks=1061440001_378456007_2_0_0__124270&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1,243 lei</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Tomis Garden Bucuresti</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/tomis-garden-bucuresti.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuALrrKDKBsACAdICJDNkMWFmYTZkLWJhN2UtNDE5MS04NmIwLTAxNjk5OTM2NmQzMNgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-01-07&amp;checkout=2026-01-10&amp;dest_id=-1153951&amp;dest_type=city&amp;group_adults=2&amp;req_adults=2&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=22&amp;hapos=22&amp;sr_order=popularity&amp;srpvid=304c7af7f14d7d22b74caeec5251d628&amp;srepoch=1766488749&amp;all_sr_blocks=0_0_2_0_0&amp;highlighted_blocks=0_0_2_0_0&amp;matching_block_id=0_0_2_0_0&amp;sr_pri_blocks=0_0_2_0_0__137193&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9.4</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Bucharest Premium Luxury Studios &amp; Apartments by Glam Story</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/bucharest-premium-luxury-studios-amp-apartments-by-glam-story.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuALrrKDKBsACAdICJDNkMWFmYTZkLWJhN2UtNDE5MS04NmIwLTAxNjk5OTM2NmQzMNgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-01-07&amp;checkout=2026-01-10&amp;dest_id=-1153951&amp;dest_type=city&amp;group_adults=2&amp;req_adults=2&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=23&amp;hapos=23&amp;sr_order=popularity&amp;srpvid=304c7af7f14d7d22b74caeec5251d628&amp;srepoch=1766488749&amp;all_sr_blocks=1337095501_412223728_2_0_0&amp;highlighted_blocks=1337095501_412223728_2_0_0&amp;matching_block_id=1337095501_412223728_2_0_0&amp;sr_pri_blocks=1337095501_412223728_2_0_0__110000&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Bright and cozy apartment in the Bucharest center</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/bright-and-cozy-apartment-in-the-bucharest-center.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuALrrKDKBsACAdICJDNkMWFmYTZkLWJhN2UtNDE5MS04NmIwLTAxNjk5OTM2NmQzMNgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-01-07&amp;checkout=2026-01-10&amp;dest_id=-1153951&amp;dest_type=city&amp;group_adults=2&amp;req_adults=2&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=24&amp;hapos=24&amp;sr_order=popularity&amp;srpvid=304c7af7f14d7d22b74caeec5251d628&amp;srepoch=1766488749&amp;all_sr_blocks=1357898201_408129470_2_0_0&amp;highlighted_blocks=1357898201_408129470_2_0_0&amp;matching_block_id=1357898201_408129470_2_0_0&amp;sr_pri_blocks=1357898201_408129470_2_0_0__58320&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>7.6</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ROSETTI Hotel</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/rosetti-aparthotel.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuALrrKDKBsACAdICJDNkMWFmYTZkLWJhN2UtNDE5MS04NmIwLTAxNjk5OTM2NmQzMNgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-01-07&amp;checkout=2026-01-10&amp;dest_id=-1153951&amp;dest_type=city&amp;group_adults=2&amp;req_adults=2&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=25&amp;hapos=25&amp;sr_order=popularity&amp;srpvid=304c7af7f14d7d22b74caeec5251d628&amp;srepoch=1766488749&amp;all_sr_blocks=0_0_2_0_0&amp;highlighted_blocks=0_0_2_0_0&amp;matching_block_id=0_0_2_0_0&amp;sr_pri_blocks=0_0_2_0_0__122275&amp;from=searchresults</x:t>
+    <x:t>2,231 lei</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Brasov Gondola Apartments</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/mgi-studio-coresi.html?label=gen173nr-10CAEoggI46AdIM1gEaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBqAIBuAK0qKrKBsACAdICJDA3Yjg3ODMzLWFlNmYtNDVmMi04NDkwLWQyOWNlZDU1NTgyYtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=2&amp;hapos=2&amp;sr_order=popularity&amp;srpvid=f0df5c6391330050&amp;srepoch=1766495350&amp;all_sr_blocks=1413131701_413051882_0_0_0&amp;highlighted_blocks=1413131701_413051882_0_0_0&amp;matching_block_id=1413131701_413051882_0_0_0&amp;sr_pri_blocks=1413131701_413051882_0_0_0__1119300&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>30,461 lei</x:t>
+  </x:si>
+  <x:si>
+    <x:t>14,888 lei</x:t>
+  </x:si>
+  <x:si>
+    <x:t>30,849 lei</x:t>
+  </x:si>
+  <x:si>
+    <x:t>40,519 lei</x:t>
+  </x:si>
+  <x:si>
+    <x:t>23,232 lei</x:t>
+  </x:si>
+  <x:si>
+    <x:t>33,443 lei</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -604,7 +658,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:D26"/>
+  <x:dimension ref="A1:C26"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:4">
@@ -623,128 +677,128 @@
     </x:row>
     <x:row r="2" spans="1:4">
       <x:c r="A2" s="0" t="s">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="B2" s="0" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B2" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
       <x:c r="C2" s="0" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="D2" s="0" t="s">
         <x:v>6</x:v>
-      </x:c>
-      <x:c r="D2" s="0" t="s">
-        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:4">
       <x:c r="A3" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B3" s="0" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="s">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B3" s="0" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="C3" s="0" t="s">
-        <x:v>10</x:v>
-      </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:4">
       <x:c r="A4" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>92</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:4">
       <x:c r="A5" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>18</x:v>
+        <x:v>93</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:4">
       <x:c r="A6" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B6" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C6" s="0" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="B6" s="0" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="C6" s="0" t="s">
-        <x:v>21</x:v>
-      </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>94</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:4">
       <x:c r="A7" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
-        <x:v>24</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C7" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
-        <x:v>25</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:4">
       <x:c r="A8" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="B8" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C8" s="0" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="D8" s="0" t="s">
         <x:v>26</x:v>
-      </x:c>
-      <x:c r="B8" s="0" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="C8" s="0" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="D8" s="0" t="s">
-        <x:v>28</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:4">
       <x:c r="A9" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B9" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="B9" s="0" t="s">
+      <x:c r="C9" s="0" t="s">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="C9" s="0" t="s">
-        <x:v>31</x:v>
-      </x:c>
       <x:c r="D9" s="0" t="s">
-        <x:v>32</x:v>
+        <x:v>23</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:4">
       <x:c r="A10" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="B10" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="C10" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="D10" s="0" t="s">
         <x:v>33</x:v>
-      </x:c>
-      <x:c r="B10" s="0" t="s">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="C10" s="0" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="D10" s="0" t="s">
-        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:4">
@@ -755,24 +809,24 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="C11" s="0" t="s">
-        <x:v>31</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D11" s="0" t="s">
-        <x:v>32</x:v>
+        <x:v>37</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:4">
       <x:c r="A12" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="B12" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="C12" s="0" t="s">
-        <x:v>39</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="D12" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>95</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:4">
@@ -786,7 +840,7 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="D13" s="0" t="s">
-        <x:v>44</x:v>
+        <x:v>96</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:4">
@@ -797,178 +851,192 @@
         <x:v>46</x:v>
       </x:c>
       <x:c r="C14" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="D14" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>97</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:4">
       <x:c r="A15" s="0" t="s">
-        <x:v>47</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="B15" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C15" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="D15" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>51</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:4">
       <x:c r="A16" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="B16" s="0" t="s">
-        <x:v>51</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="C16" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="D16" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>54</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:4">
       <x:c r="A17" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="B17" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="C17" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="D17" s="0" t="s">
-        <x:v>55</x:v>
+        <x:v>34</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:4">
       <x:c r="A18" s="0" t="s">
-        <x:v>56</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="B18" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="C18" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="D18" s="0" t="s">
-        <x:v>55</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:4">
       <x:c r="A19" s="0" t="s">
-        <x:v>59</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="B19" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="C19" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="D19" s="0" t="s">
-        <x:v>62</x:v>
+        <x:v>63</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:4">
       <x:c r="A20" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="B20" s="0" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="C20" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="D20" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>27</x:v>
       </x:c>
     </x:row>
     <x:row r="21" spans="1:4">
       <x:c r="A21" s="0" t="s">
-        <x:v>65</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="B21" s="0" t="s">
-        <x:v>66</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C21" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="D21" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>68</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:4">
       <x:c r="A22" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="B22" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="C22" s="0" t="s">
         <x:v>69</x:v>
       </x:c>
       <x:c r="D22" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>72</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:4">
       <x:c r="A23" s="0" t="s">
-        <x:v>70</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="B23" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="C23" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="D23" s="0" t="s">
-        <x:v>72</x:v>
+        <x:v>48</x:v>
       </x:c>
     </x:row>
     <x:row r="24" spans="1:4">
       <x:c r="A24" s="0" t="s">
-        <x:v>73</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="B24" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="C24" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D24" s="0" t="s">
-        <x:v>32</x:v>
+        <x:v>78</x:v>
       </x:c>
     </x:row>
     <x:row r="25" spans="1:4">
       <x:c r="A25" s="0" t="s">
-        <x:v>75</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="B25" s="0" t="s">
-        <x:v>76</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="C25" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D25" s="0" t="s">
-        <x:v>77</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="26" spans="1:4">
       <x:c r="A26" s="0" t="s">
-        <x:v>78</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="B26" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="C26" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="D26" s="0" t="s">
-        <x:v>18</x:v>
+        <x:v>82</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" spans="1:4">
+      <x:c r="A27" s="0" t="s">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="B27" s="0" t="s">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="C27" s="0" t="s">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="D27" s="0" t="s">
+        <x:v>89</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>